<commit_message>
Prepare bilingual development preview and Connect deployments
</commit_message>
<xml_diff>
--- a/data-raw/languages.xlsx
+++ b/data-raw/languages.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2469" uniqueCount="2469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2471" uniqueCount="2471">
   <si>
     <t>Deutsch</t>
   </si>
@@ -7422,6 +7422,12 @@
   </si>
   <si>
     <t xml:space="preserve">Archivierte Tabelle der Änderungen von Wirkfaktoren und DER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://litg-spectran-en.share.connect.posit.cloud/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://litg-spectran-de.share.connect.posit.cloud/</t>
   </si>
 </sst>
 </file>
@@ -8059,10 +8065,10 @@
         <v>lang$global(14)</v>
       </c>
       <c r="D15" t="s">
-        <v>617</v>
+        <v>2469</v>
       </c>
       <c r="E15" t="s">
-        <v>616</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="16">

</xml_diff>